<commit_message>
feat(wnba): scrape today's slate (875 props), refresh 2026-05-06 graded JSON, add slate_sport_wnba.json artifact
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-06.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-06.xlsx
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2551</v>
+        <v>2561</v>
       </c>
       <c r="E17" t="n">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F17" t="n">
-        <v>2020</v>
+        <v>2029</v>
       </c>
       <c r="G17" t="n">
         <v>20.8</v>
@@ -1451,8 +1451,11 @@
       <c r="O6" t="n">
         <v>0</v>
       </c>
+      <c r="P6" t="n">
+        <v>10</v>
+      </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -1531,7 +1534,7 @@
         <v>20.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>2551</v>
+        <v>2561</v>
       </c>
       <c r="R7" t="n">
         <v>50</v>

</xml_diff>